<commit_message>
Add FY cost avoidance chart to September 2026 metrics workbook
Adds two sheets without changing the Metrics sheet or its existing charts:
- 'FY Chart': combo chart of monthly cost avoidance (columns, left axis)
  with FY22-FY25 totals (labeled markers) and FY26/FY27 running totals
  (lines, right axis), Oct 2021 - Sep 2027.
- 'FY Chart Data': formula-driven helper table pulling Metrics row 32 by
  month (DoD fiscal year, Oct-Sep) plus an FY summary. FY27 months are
  pre-built and extend automatically as months are added to Metrics.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RqKSyuPB2tSMQAr5eSeDK8
</commit_message>
<xml_diff>
--- a/OFFLINE_September 2026 Cost Avoidance Metrics.xlsx
+++ b/OFFLINE_September 2026 Cost Avoidance Metrics.xlsx
@@ -14,11 +14,14 @@
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
+    <sheet name="FY Chart" sheetId="2" r:id="rId101"/>
+    <sheet name="FY Chart Data" sheetId="3" r:id="rId102"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$AO$1:$AO$32</definedName>
+    <definedName name="FY27_RunningTotal" localSheetId="2">OFFSET('FY Chart Data'!$G$5,0,0,60+COUNTIF('FY Chart Data'!$C$65:$C$76,"Yes"),1)</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -140,7 +143,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +167,22 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF52514E"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -275,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -333,6 +352,20 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4496,6 +4529,1809 @@
     <c:pageSetup/>
   </c:printSettings>
   <c:userShapes r:id="rId3"/>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1600" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1600" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0B0B0B"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Cost Avoidance by Month and Fiscal Year (FY22 - FY27)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'FY Chart Data'!$D$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Monthly Cost Avoidance</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$A$5:$A$76</c:f>
+              <c:numCache>
+                <c:formatCode>mmm-yy</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="0">
+                  <c:v>44470</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44531</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44562</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44593</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44621</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44652</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44682</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44713</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44743</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44774</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44805</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44835</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44866</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44896</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44927</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44958</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44986</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>45017</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>45047</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>45078</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>45108</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>45139</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>45170</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>45200</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>45231</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>45261</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>45292</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>45323</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>45352</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45536</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>45566</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>45597</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>45627</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>45658</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>45689</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>45717</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>45748</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45778</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45809</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45839</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>45870</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>45901</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>45931</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>45962</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>45992</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>46023</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>46054</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>46082</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>46113</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>46143</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>46235</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>46296</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>46327</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>46357</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>46388</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>46419</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>46447</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>46478</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>46508</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>46539</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>46569</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>46600</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>46631</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$D$5:$D$76</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="0">
+                  <c:v>658056</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1385814</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>827246</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>486420</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>893075</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>510498</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>541754</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>302936</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>424822</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2400958</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3126402</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1293912</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2502625</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1465528</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>732107</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1109014</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>578484</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>704828</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1929683</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1457159</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>76884</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>259452</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>676463</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>337750</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>115182</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>448861</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>643129</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>2091106</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>766513</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>188087</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>874601</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2869690</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1840432</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2957414</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>3109264</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2372898</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1713238</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>1020464</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>1382141</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>834311</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>1039025</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>1749951</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>977319</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>1455812</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>1136435</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>1682848</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>3062808</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>2882896</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>2105658</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>2542368</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>3443673</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>1382386</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>2048749</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>2610208</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>2248040</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>1772218</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>2332123</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>2450656</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>3524184</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>2286606</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="35"/>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'FY Chart Data'!$E$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>FY Total (FY22-FY25)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="11"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="3D3C3A"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:ln w="6350">
+                <a:solidFill>
+                  <a:srgbClr val="BFBFBF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$A$5:$A$76</c:f>
+              <c:numCache>
+                <c:formatCode>mmm-yy</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="0">
+                  <c:v>44470</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44531</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44562</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44593</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44621</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44652</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44682</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44713</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44743</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44774</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44805</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44835</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44866</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44896</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44927</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44958</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44986</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>45017</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>45047</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>45078</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>45108</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>45139</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>45170</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>45200</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>45231</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>45261</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>45292</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>45323</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>45352</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45536</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>45566</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>45597</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>45627</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>45658</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>45689</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>45717</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>45748</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45778</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45809</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45839</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>45870</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>45901</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>45931</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>45962</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>45992</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>46023</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>46054</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>46082</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>46113</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>46143</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>46235</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>46296</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>46327</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>46357</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>46388</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>46419</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>46447</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>46478</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>46508</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>46539</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>46569</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>46600</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>46631</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$E$5:$E$76</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="11">
+                  <c:v>12851893</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>11829977</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>15904279</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>18427250</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'FY Chart Data'!$H$5:$H$76</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="72"/>
+                  <c:pt idx="11">
+                    <c:v>FY22 Total: $12.9M</c:v>
+                  </c:pt>
+                  <c:pt idx="23">
+                    <c:v>FY23 Total: $11.8M</c:v>
+                  </c:pt>
+                  <c:pt idx="35">
+                    <c:v>FY24 Total: $15.9M</c:v>
+                  </c:pt>
+                  <c:pt idx="47">
+                    <c:v>FY25 Total: $18.4M</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'FY Chart Data'!$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>FY26 Running Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:ln w="6350">
+                <a:solidFill>
+                  <a:srgbClr val="BFBFBF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$A$5:$A$76</c:f>
+              <c:numCache>
+                <c:formatCode>mmm-yy</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="0">
+                  <c:v>44470</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44531</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44562</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44593</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44621</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44652</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44682</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44713</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44743</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44774</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44805</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44835</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44866</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44896</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44927</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44958</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44986</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>45017</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>45047</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>45078</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>45108</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>45139</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>45170</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>45200</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>45231</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>45261</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>45292</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>45323</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>45352</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45536</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>45566</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>45597</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>45627</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>45658</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>45689</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>45717</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>45748</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45778</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45809</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45839</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>45870</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>45901</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>45931</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>45962</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>45992</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>46023</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>46054</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>46082</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>46113</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>46143</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>46235</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>46296</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>46327</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>46357</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>46388</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>46419</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>46447</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>46478</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>46508</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>46539</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>46569</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>46600</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>46631</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$F$5:$F$76</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="48">
+                  <c:v>2882896</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>4988554</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>7530922</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>10974595</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>12356981</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>14405730</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>17015938</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>19263978</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>21036196</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>23368319</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>25818975</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>29343159</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'FY Chart Data'!$I$5:$I$76</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="72"/>
+                  <c:pt idx="59">
+                    <c:v>FY26 Running Total: $29.3M (thru Sep-26)</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'FY Chart Data'!$G$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>FY27 Running Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:ln w="6350">
+                <a:solidFill>
+                  <a:srgbClr val="BFBFBF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="0B0B0B"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showDataLabelsRange val="1"/>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'FY Chart Data'!$A$5:$A$76</c:f>
+              <c:numCache>
+                <c:formatCode>mmm-yy</c:formatCode>
+                <c:ptCount val="72"/>
+                <c:pt idx="0">
+                  <c:v>44470</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>44501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>44531</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44562</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>44593</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>44621</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>44652</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>44682</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44713</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>44743</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>44774</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44805</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>44835</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>44866</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>44896</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>44927</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>44958</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>44986</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>45017</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>45047</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>45078</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>45108</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>45139</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>45170</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>45200</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>45231</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>45261</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>45292</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>45323</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>45352</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>45536</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>45566</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>45597</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>45627</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>45658</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>45689</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>45717</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>45748</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>45778</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45809</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>45839</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>45870</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>45901</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>45931</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>45962</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>45992</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>46023</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>46054</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>46082</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>46113</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>46143</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>46235</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>46266</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>46296</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>46327</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>46357</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>46388</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>46419</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>46447</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>46478</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>46508</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>46539</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>46569</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>46600</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>46631</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'FY Chart Data'!FY27_RunningTotal</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0</c:formatCode>
+                <c:ptCount val="61"/>
+                <c:pt idx="60">
+                  <c:v>2286606</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+              <c15:datalabelsRange>
+                <c15:f>'FY Chart Data'!$J$5:$J$76</c15:f>
+                <c15:dlblRangeCache>
+                  <c:ptCount val="72"/>
+                  <c:pt idx="60">
+                    <c:v>FY27 Running Total: $2.3M (thru Oct-26)</c:v>
+                  </c:pt>
+                </c15:dlblRangeCache>
+              </c15:datalabelsRange>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="50010003"/>
+        <c:axId val="50010004"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm\-yy" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="BFBFBF"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-5400000" vert="horz"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="800" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52514E"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="0"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickLblSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E5E5E3"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="52514E"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="52514E"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Monthly Cost Avoidance (columns)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="&quot;$&quot;#,##0.0,,&quot;M&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52514E"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="50010003"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm\-yy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010004"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="0"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010004"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="52514E"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1100" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="52514E"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>FY Total / Running Total (diamonds &amp; lines)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="&quot;$&quot;#,##0.0,,&quot;M&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52514E"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50010003"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1000" b="0">
+              <a:solidFill>
+                <a:srgbClr val="0B0B0B"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:latin typeface="Calibri"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup orientation="landscape"/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
@@ -5827,6 +7663,41 @@
 </c:userShapes>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="FY Cost Avoidance Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -20090,6 +21961,1769 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source: 'FY Chart Data' sheet (formulas pulling from Metrics row 32). DoD fiscal year, Oct 1 - Sep 30. Columns = monthly cost avoidance (left axis). Diamonds = completed-FY totals; lines = FY26 and FY27 running totals (right axis).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O76"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="3" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="26" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY Cost Avoidance Chart Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeds the 'FY Chart' sheet. Every value is a formula that pulls from Metrics row 32 (Volume of Cost Avoidance), matched by month using the Metrics row 25 dates. Do not type over these cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiscal year = DoD fiscal year: Oct 1 - Sep 30, named for the year it ends (FY26 = Oct 2025 - Sep 2026). A5 (Oct-21) is the only typed value; FY27 months are pre-built and fill in as months are added to Metrics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Month</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiscal Year</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Month Reported?</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monthly Cost Avoidance</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY Total (FY22-FY25)</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY26 Running Total</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY27 Running Total</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY Total Label</t>
+        </is>
+      </c>
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY26 Label</t>
+        </is>
+      </c>
+      <c r="J4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY27 Label</t>
+        </is>
+      </c>
+      <c r="L4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fiscal Year</t>
+        </is>
+      </c>
+      <c r="M4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Months Reported</t>
+        </is>
+      </c>
+      <c r="N4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY Total Cost Avoidance</t>
+        </is>
+      </c>
+      <c r="O4" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28">
+        <v>44470</v>
+      </c>
+      <c r="B5" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A5)+IF(MONTH(A5)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C5" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A5,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A5),MONTH(A5)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D5" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A5,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A5),MONTH(A5)+1,1))</f>
+        <v>658056</v>
+      </c>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY22</t>
+        </is>
+      </c>
+      <c r="M5" s="29">
+        <f>COUNTIFS($B$5:$B$76,L5,$C$5:$C$76,"Yes")</f>
+        <v>12</v>
+      </c>
+      <c r="N5" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L5)</f>
+        <v>12851893</v>
+      </c>
+      <c r="O5" s="31" t="str">
+        <f>IF(M5=12,"Complete","In progress ("&amp;M5&amp;" of 12 months)")</f>
+        <v>Complete</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28">
+        <f>DATE(YEAR(A5),MONTH(A5)+1,1)</f>
+        <v>44501</v>
+      </c>
+      <c r="B6" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A6)+IF(MONTH(A6)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C6" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A6,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A6),MONTH(A6)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D6" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A6,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A6),MONTH(A6)+1,1))</f>
+        <v>1385814</v>
+      </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY23</t>
+        </is>
+      </c>
+      <c r="M6" s="29">
+        <f>COUNTIFS($B$5:$B$76,L6,$C$5:$C$76,"Yes")</f>
+        <v>12</v>
+      </c>
+      <c r="N6" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L6)</f>
+        <v>11829977</v>
+      </c>
+      <c r="O6" s="31" t="str">
+        <f>IF(M6=12,"Complete","In progress ("&amp;M6&amp;" of 12 months)")</f>
+        <v>Complete</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28">
+        <f>DATE(YEAR(A6),MONTH(A6)+1,1)</f>
+        <v>44531</v>
+      </c>
+      <c r="B7" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A7)+IF(MONTH(A7)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C7" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A7,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A7),MONTH(A7)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D7" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A7,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A7),MONTH(A7)+1,1))</f>
+        <v>827246</v>
+      </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY24</t>
+        </is>
+      </c>
+      <c r="M7" s="29">
+        <f>COUNTIFS($B$5:$B$76,L7,$C$5:$C$76,"Yes")</f>
+        <v>12</v>
+      </c>
+      <c r="N7" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L7)</f>
+        <v>15904279</v>
+      </c>
+      <c r="O7" s="31" t="str">
+        <f>IF(M7=12,"Complete","In progress ("&amp;M7&amp;" of 12 months)")</f>
+        <v>Complete</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28">
+        <f>DATE(YEAR(A7),MONTH(A7)+1,1)</f>
+        <v>44562</v>
+      </c>
+      <c r="B8" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A8)+IF(MONTH(A8)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C8" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A8,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A8),MONTH(A8)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D8" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A8,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A8),MONTH(A8)+1,1))</f>
+        <v>486420</v>
+      </c>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY25</t>
+        </is>
+      </c>
+      <c r="M8" s="29">
+        <f>COUNTIFS($B$5:$B$76,L8,$C$5:$C$76,"Yes")</f>
+        <v>12</v>
+      </c>
+      <c r="N8" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L8)</f>
+        <v>18427250</v>
+      </c>
+      <c r="O8" s="31" t="str">
+        <f>IF(M8=12,"Complete","In progress ("&amp;M8&amp;" of 12 months)")</f>
+        <v>Complete</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28">
+        <f>DATE(YEAR(A8),MONTH(A8)+1,1)</f>
+        <v>44593</v>
+      </c>
+      <c r="B9" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A9)+IF(MONTH(A9)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C9" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A9,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A9),MONTH(A9)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D9" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A9,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A9),MONTH(A9)+1,1))</f>
+        <v>893075</v>
+      </c>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY26</t>
+        </is>
+      </c>
+      <c r="M9" s="29">
+        <f>COUNTIFS($B$5:$B$76,L9,$C$5:$C$76,"Yes")</f>
+        <v>12</v>
+      </c>
+      <c r="N9" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L9)</f>
+        <v>29343159</v>
+      </c>
+      <c r="O9" s="31" t="str">
+        <f>IF(M9=12,"Complete","In progress ("&amp;M9&amp;" of 12 months)")</f>
+        <v>Complete</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28">
+        <f>DATE(YEAR(A9),MONTH(A9)+1,1)</f>
+        <v>44621</v>
+      </c>
+      <c r="B10" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A10)+IF(MONTH(A10)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C10" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A10,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A10),MONTH(A10)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D10" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A10,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A10),MONTH(A10)+1,1))</f>
+        <v>510498</v>
+      </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY27</t>
+        </is>
+      </c>
+      <c r="M10" s="29">
+        <f>COUNTIFS($B$5:$B$76,L10,$C$5:$C$76,"Yes")</f>
+        <v>1</v>
+      </c>
+      <c r="N10" s="32">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,L10)</f>
+        <v>2286606</v>
+      </c>
+      <c r="O10" s="31" t="str">
+        <f>IF(M10=12,"Complete","In progress ("&amp;M10&amp;" of 12 months)")</f>
+        <v>In progress (1 of 12 months)</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28">
+        <f>DATE(YEAR(A10),MONTH(A10)+1,1)</f>
+        <v>44652</v>
+      </c>
+      <c r="B11" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A11)+IF(MONTH(A11)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C11" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A11,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A11),MONTH(A11)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D11" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A11,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A11),MONTH(A11)+1,1))</f>
+        <v>541754</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28">
+        <f>DATE(YEAR(A11),MONTH(A11)+1,1)</f>
+        <v>44682</v>
+      </c>
+      <c r="B12" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A12)+IF(MONTH(A12)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C12" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A12,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A12),MONTH(A12)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D12" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A12,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A12),MONTH(A12)+1,1))</f>
+        <v>302936</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28">
+        <f>DATE(YEAR(A12),MONTH(A12)+1,1)</f>
+        <v>44713</v>
+      </c>
+      <c r="B13" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A13)+IF(MONTH(A13)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C13" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A13,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A13),MONTH(A13)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D13" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A13,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A13),MONTH(A13)+1,1))</f>
+        <v>424822</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28">
+        <f>DATE(YEAR(A13),MONTH(A13)+1,1)</f>
+        <v>44743</v>
+      </c>
+      <c r="B14" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A14)+IF(MONTH(A14)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C14" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A14,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A14),MONTH(A14)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D14" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A14,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A14),MONTH(A14)+1,1))</f>
+        <v>2400958</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28">
+        <f>DATE(YEAR(A14),MONTH(A14)+1,1)</f>
+        <v>44774</v>
+      </c>
+      <c r="B15" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A15)+IF(MONTH(A15)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C15" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A15,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A15),MONTH(A15)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D15" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A15,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A15),MONTH(A15)+1,1))</f>
+        <v>3126402</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28">
+        <f>DATE(YEAR(A15),MONTH(A15)+1,1)</f>
+        <v>44805</v>
+      </c>
+      <c r="B16" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A16)+IF(MONTH(A16)&gt;=10,1,0),2)</f>
+        <v>FY22</v>
+      </c>
+      <c r="C16" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A16,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A16),MONTH(A16)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D16" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A16,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A16),MONTH(A16)+1,1))</f>
+        <v>1293912</v>
+      </c>
+      <c r="E16" s="30">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,B16)</f>
+        <v>12851893</v>
+      </c>
+      <c r="H16" s="31" t="str">
+        <f>B16&amp;" Total: "&amp;TEXT(E16,"$0.0,,")&amp;"M"</f>
+        <v>FY22 Total: $12.9M</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28">
+        <f>DATE(YEAR(A16),MONTH(A16)+1,1)</f>
+        <v>44835</v>
+      </c>
+      <c r="B17" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A17)+IF(MONTH(A17)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C17" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A17,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A17),MONTH(A17)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D17" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A17,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A17),MONTH(A17)+1,1))</f>
+        <v>2502625</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28">
+        <f>DATE(YEAR(A17),MONTH(A17)+1,1)</f>
+        <v>44866</v>
+      </c>
+      <c r="B18" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A18)+IF(MONTH(A18)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C18" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A18,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A18),MONTH(A18)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D18" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A18,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A18),MONTH(A18)+1,1))</f>
+        <v>1465528</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28">
+        <f>DATE(YEAR(A18),MONTH(A18)+1,1)</f>
+        <v>44896</v>
+      </c>
+      <c r="B19" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A19)+IF(MONTH(A19)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C19" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A19,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A19),MONTH(A19)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D19" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A19,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A19),MONTH(A19)+1,1))</f>
+        <v>732107</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28">
+        <f>DATE(YEAR(A19),MONTH(A19)+1,1)</f>
+        <v>44927</v>
+      </c>
+      <c r="B20" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A20)+IF(MONTH(A20)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C20" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A20,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A20),MONTH(A20)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D20" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A20,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A20),MONTH(A20)+1,1))</f>
+        <v>1109014</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28">
+        <f>DATE(YEAR(A20),MONTH(A20)+1,1)</f>
+        <v>44958</v>
+      </c>
+      <c r="B21" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A21)+IF(MONTH(A21)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C21" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A21,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A21),MONTH(A21)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D21" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A21,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A21),MONTH(A21)+1,1))</f>
+        <v>578484</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28">
+        <f>DATE(YEAR(A21),MONTH(A21)+1,1)</f>
+        <v>44986</v>
+      </c>
+      <c r="B22" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A22)+IF(MONTH(A22)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C22" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A22,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A22),MONTH(A22)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D22" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A22,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A22),MONTH(A22)+1,1))</f>
+        <v>704828</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28">
+        <f>DATE(YEAR(A22),MONTH(A22)+1,1)</f>
+        <v>45017</v>
+      </c>
+      <c r="B23" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A23)+IF(MONTH(A23)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C23" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A23,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A23),MONTH(A23)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D23" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A23,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A23),MONTH(A23)+1,1))</f>
+        <v>1929683</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28">
+        <f>DATE(YEAR(A23),MONTH(A23)+1,1)</f>
+        <v>45047</v>
+      </c>
+      <c r="B24" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A24)+IF(MONTH(A24)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C24" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A24,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A24),MONTH(A24)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D24" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A24,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A24),MONTH(A24)+1,1))</f>
+        <v>1457159</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28">
+        <f>DATE(YEAR(A24),MONTH(A24)+1,1)</f>
+        <v>45078</v>
+      </c>
+      <c r="B25" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A25)+IF(MONTH(A25)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C25" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A25,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A25),MONTH(A25)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D25" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A25,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A25),MONTH(A25)+1,1))</f>
+        <v>76884</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28">
+        <f>DATE(YEAR(A25),MONTH(A25)+1,1)</f>
+        <v>45108</v>
+      </c>
+      <c r="B26" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A26)+IF(MONTH(A26)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C26" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A26,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A26),MONTH(A26)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D26" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A26,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A26),MONTH(A26)+1,1))</f>
+        <v>259452</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28">
+        <f>DATE(YEAR(A26),MONTH(A26)+1,1)</f>
+        <v>45139</v>
+      </c>
+      <c r="B27" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A27)+IF(MONTH(A27)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C27" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A27,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A27),MONTH(A27)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D27" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A27,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A27),MONTH(A27)+1,1))</f>
+        <v>676463</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28">
+        <f>DATE(YEAR(A27),MONTH(A27)+1,1)</f>
+        <v>45170</v>
+      </c>
+      <c r="B28" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A28)+IF(MONTH(A28)&gt;=10,1,0),2)</f>
+        <v>FY23</v>
+      </c>
+      <c r="C28" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A28,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A28),MONTH(A28)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D28" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A28,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A28),MONTH(A28)+1,1))</f>
+        <v>337750</v>
+      </c>
+      <c r="E28" s="30">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,B28)</f>
+        <v>11829977</v>
+      </c>
+      <c r="H28" s="31" t="str">
+        <f>B28&amp;" Total: "&amp;TEXT(E28,"$0.0,,")&amp;"M"</f>
+        <v>FY23 Total: $11.8M</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="28">
+        <f>DATE(YEAR(A28),MONTH(A28)+1,1)</f>
+        <v>45200</v>
+      </c>
+      <c r="B29" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A29)+IF(MONTH(A29)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C29" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A29,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A29),MONTH(A29)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D29" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A29,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A29),MONTH(A29)+1,1))</f>
+        <v>115182</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="28">
+        <f>DATE(YEAR(A29),MONTH(A29)+1,1)</f>
+        <v>45231</v>
+      </c>
+      <c r="B30" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A30)+IF(MONTH(A30)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C30" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A30,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A30),MONTH(A30)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D30" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A30,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A30),MONTH(A30)+1,1))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28">
+        <f>DATE(YEAR(A30),MONTH(A30)+1,1)</f>
+        <v>45261</v>
+      </c>
+      <c r="B31" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A31)+IF(MONTH(A31)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C31" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A31,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A31),MONTH(A31)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D31" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A31,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A31),MONTH(A31)+1,1))</f>
+        <v>448861</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28">
+        <f>DATE(YEAR(A31),MONTH(A31)+1,1)</f>
+        <v>45292</v>
+      </c>
+      <c r="B32" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A32)+IF(MONTH(A32)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C32" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A32,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A32),MONTH(A32)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D32" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A32,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A32),MONTH(A32)+1,1))</f>
+        <v>643129</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28">
+        <f>DATE(YEAR(A32),MONTH(A32)+1,1)</f>
+        <v>45323</v>
+      </c>
+      <c r="B33" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A33)+IF(MONTH(A33)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C33" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A33,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A33),MONTH(A33)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D33" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A33,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A33),MONTH(A33)+1,1))</f>
+        <v>2091106</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="28">
+        <f>DATE(YEAR(A33),MONTH(A33)+1,1)</f>
+        <v>45352</v>
+      </c>
+      <c r="B34" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A34)+IF(MONTH(A34)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C34" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A34,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A34),MONTH(A34)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D34" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A34,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A34),MONTH(A34)+1,1))</f>
+        <v>766513</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28">
+        <f>DATE(YEAR(A34),MONTH(A34)+1,1)</f>
+        <v>45383</v>
+      </c>
+      <c r="B35" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A35)+IF(MONTH(A35)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C35" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A35,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A35),MONTH(A35)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D35" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A35,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A35),MONTH(A35)+1,1))</f>
+        <v>188087</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28">
+        <f>DATE(YEAR(A35),MONTH(A35)+1,1)</f>
+        <v>45413</v>
+      </c>
+      <c r="B36" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A36)+IF(MONTH(A36)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C36" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A36,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A36),MONTH(A36)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D36" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A36,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A36),MONTH(A36)+1,1))</f>
+        <v>874601</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="28">
+        <f>DATE(YEAR(A36),MONTH(A36)+1,1)</f>
+        <v>45444</v>
+      </c>
+      <c r="B37" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A37)+IF(MONTH(A37)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C37" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A37,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A37),MONTH(A37)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D37" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A37,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A37),MONTH(A37)+1,1))</f>
+        <v>2869690</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="28">
+        <f>DATE(YEAR(A37),MONTH(A37)+1,1)</f>
+        <v>45474</v>
+      </c>
+      <c r="B38" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A38)+IF(MONTH(A38)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C38" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A38,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A38),MONTH(A38)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D38" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A38,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A38),MONTH(A38)+1,1))</f>
+        <v>1840432</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="28">
+        <f>DATE(YEAR(A38),MONTH(A38)+1,1)</f>
+        <v>45505</v>
+      </c>
+      <c r="B39" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A39)+IF(MONTH(A39)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C39" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A39,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A39),MONTH(A39)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D39" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A39,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A39),MONTH(A39)+1,1))</f>
+        <v>2957414</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="28">
+        <f>DATE(YEAR(A39),MONTH(A39)+1,1)</f>
+        <v>45536</v>
+      </c>
+      <c r="B40" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A40)+IF(MONTH(A40)&gt;=10,1,0),2)</f>
+        <v>FY24</v>
+      </c>
+      <c r="C40" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A40,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A40),MONTH(A40)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D40" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A40,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A40),MONTH(A40)+1,1))</f>
+        <v>3109264</v>
+      </c>
+      <c r="E40" s="30">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,B40)</f>
+        <v>15904279</v>
+      </c>
+      <c r="H40" s="31" t="str">
+        <f>B40&amp;" Total: "&amp;TEXT(E40,"$0.0,,")&amp;"M"</f>
+        <v>FY24 Total: $15.9M</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="28">
+        <f>DATE(YEAR(A40),MONTH(A40)+1,1)</f>
+        <v>45566</v>
+      </c>
+      <c r="B41" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A41)+IF(MONTH(A41)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C41" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A41,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A41),MONTH(A41)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D41" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A41,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A41),MONTH(A41)+1,1))</f>
+        <v>2372898</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="28">
+        <f>DATE(YEAR(A41),MONTH(A41)+1,1)</f>
+        <v>45597</v>
+      </c>
+      <c r="B42" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A42)+IF(MONTH(A42)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C42" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A42,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A42),MONTH(A42)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D42" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A42,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A42),MONTH(A42)+1,1))</f>
+        <v>1713238</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28">
+        <f>DATE(YEAR(A42),MONTH(A42)+1,1)</f>
+        <v>45627</v>
+      </c>
+      <c r="B43" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A43)+IF(MONTH(A43)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C43" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A43,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A43),MONTH(A43)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D43" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A43,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A43),MONTH(A43)+1,1))</f>
+        <v>1020464</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="28">
+        <f>DATE(YEAR(A43),MONTH(A43)+1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="B44" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A44)+IF(MONTH(A44)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C44" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A44,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A44),MONTH(A44)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D44" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A44,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A44),MONTH(A44)+1,1))</f>
+        <v>1382141</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28">
+        <f>DATE(YEAR(A44),MONTH(A44)+1,1)</f>
+        <v>45689</v>
+      </c>
+      <c r="B45" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A45)+IF(MONTH(A45)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C45" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A45,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A45),MONTH(A45)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D45" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A45,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A45),MONTH(A45)+1,1))</f>
+        <v>834311</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="28">
+        <f>DATE(YEAR(A45),MONTH(A45)+1,1)</f>
+        <v>45717</v>
+      </c>
+      <c r="B46" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A46)+IF(MONTH(A46)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C46" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A46,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A46),MONTH(A46)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D46" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A46,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A46),MONTH(A46)+1,1))</f>
+        <v>1039025</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="28">
+        <f>DATE(YEAR(A46),MONTH(A46)+1,1)</f>
+        <v>45748</v>
+      </c>
+      <c r="B47" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A47)+IF(MONTH(A47)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C47" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A47,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A47),MONTH(A47)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D47" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A47,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A47),MONTH(A47)+1,1))</f>
+        <v>1749951</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="28">
+        <f>DATE(YEAR(A47),MONTH(A47)+1,1)</f>
+        <v>45778</v>
+      </c>
+      <c r="B48" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A48)+IF(MONTH(A48)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C48" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A48,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A48),MONTH(A48)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D48" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A48,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A48),MONTH(A48)+1,1))</f>
+        <v>977319</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="28">
+        <f>DATE(YEAR(A48),MONTH(A48)+1,1)</f>
+        <v>45809</v>
+      </c>
+      <c r="B49" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A49)+IF(MONTH(A49)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C49" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A49,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A49),MONTH(A49)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D49" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A49,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A49),MONTH(A49)+1,1))</f>
+        <v>1455812</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28">
+        <f>DATE(YEAR(A49),MONTH(A49)+1,1)</f>
+        <v>45839</v>
+      </c>
+      <c r="B50" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A50)+IF(MONTH(A50)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C50" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A50,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A50),MONTH(A50)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D50" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A50,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A50),MONTH(A50)+1,1))</f>
+        <v>1136435</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="28">
+        <f>DATE(YEAR(A50),MONTH(A50)+1,1)</f>
+        <v>45870</v>
+      </c>
+      <c r="B51" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A51)+IF(MONTH(A51)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C51" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A51,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A51),MONTH(A51)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D51" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A51,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A51),MONTH(A51)+1,1))</f>
+        <v>1682848</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="28">
+        <f>DATE(YEAR(A51),MONTH(A51)+1,1)</f>
+        <v>45901</v>
+      </c>
+      <c r="B52" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A52)+IF(MONTH(A52)&gt;=10,1,0),2)</f>
+        <v>FY25</v>
+      </c>
+      <c r="C52" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A52,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A52),MONTH(A52)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D52" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A52,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A52),MONTH(A52)+1,1))</f>
+        <v>3062808</v>
+      </c>
+      <c r="E52" s="30">
+        <f>SUMIFS($D$5:$D$76,$B$5:$B$76,B52)</f>
+        <v>18427250</v>
+      </c>
+      <c r="H52" s="31" t="str">
+        <f>B52&amp;" Total: "&amp;TEXT(E52,"$0.0,,")&amp;"M"</f>
+        <v>FY25 Total: $18.4M</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="28">
+        <f>DATE(YEAR(A52),MONTH(A52)+1,1)</f>
+        <v>45931</v>
+      </c>
+      <c r="B53" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A53)+IF(MONTH(A53)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C53" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A53,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A53),MONTH(A53)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D53" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A53,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A53),MONTH(A53)+1,1))</f>
+        <v>2882896</v>
+      </c>
+      <c r="F53" s="30">
+        <f>IF(C53="Yes",D53,"")</f>
+        <v>2882896</v>
+      </c>
+      <c r="I53" s="31" t="str">
+        <f>IF(AND(C53="Yes",C54&lt;&gt;"Yes"),B53&amp;" Running Total: "&amp;TEXT(F53,"$0.0,,")&amp;"M (thru "&amp;TEXT(A53,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="28">
+        <f>DATE(YEAR(A53),MONTH(A53)+1,1)</f>
+        <v>45962</v>
+      </c>
+      <c r="B54" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A54)+IF(MONTH(A54)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C54" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A54,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A54),MONTH(A54)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D54" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A54,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A54),MONTH(A54)+1,1))</f>
+        <v>2105658</v>
+      </c>
+      <c r="F54" s="30">
+        <f>IF(C54="Yes",N(F53)+D54,"")</f>
+        <v>4988554</v>
+      </c>
+      <c r="I54" s="31" t="str">
+        <f>IF(AND(C54="Yes",C55&lt;&gt;"Yes"),B54&amp;" Running Total: "&amp;TEXT(F54,"$0.0,,")&amp;"M (thru "&amp;TEXT(A54,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="28">
+        <f>DATE(YEAR(A54),MONTH(A54)+1,1)</f>
+        <v>45992</v>
+      </c>
+      <c r="B55" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A55)+IF(MONTH(A55)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C55" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A55,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A55),MONTH(A55)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D55" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A55,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A55),MONTH(A55)+1,1))</f>
+        <v>2542368</v>
+      </c>
+      <c r="F55" s="30">
+        <f>IF(C55="Yes",N(F54)+D55,"")</f>
+        <v>7530922</v>
+      </c>
+      <c r="I55" s="31" t="str">
+        <f>IF(AND(C55="Yes",C56&lt;&gt;"Yes"),B55&amp;" Running Total: "&amp;TEXT(F55,"$0.0,,")&amp;"M (thru "&amp;TEXT(A55,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="28">
+        <f>DATE(YEAR(A55),MONTH(A55)+1,1)</f>
+        <v>46023</v>
+      </c>
+      <c r="B56" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A56)+IF(MONTH(A56)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C56" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A56,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A56),MONTH(A56)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D56" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A56,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A56),MONTH(A56)+1,1))</f>
+        <v>3443673</v>
+      </c>
+      <c r="F56" s="30">
+        <f>IF(C56="Yes",N(F55)+D56,"")</f>
+        <v>10974595</v>
+      </c>
+      <c r="I56" s="31" t="str">
+        <f>IF(AND(C56="Yes",C57&lt;&gt;"Yes"),B56&amp;" Running Total: "&amp;TEXT(F56,"$0.0,,")&amp;"M (thru "&amp;TEXT(A56,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="28">
+        <f>DATE(YEAR(A56),MONTH(A56)+1,1)</f>
+        <v>46054</v>
+      </c>
+      <c r="B57" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A57)+IF(MONTH(A57)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C57" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A57,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A57),MONTH(A57)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D57" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A57,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A57),MONTH(A57)+1,1))</f>
+        <v>1382386</v>
+      </c>
+      <c r="F57" s="30">
+        <f>IF(C57="Yes",N(F56)+D57,"")</f>
+        <v>12356981</v>
+      </c>
+      <c r="I57" s="31" t="str">
+        <f>IF(AND(C57="Yes",C58&lt;&gt;"Yes"),B57&amp;" Running Total: "&amp;TEXT(F57,"$0.0,,")&amp;"M (thru "&amp;TEXT(A57,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="28">
+        <f>DATE(YEAR(A57),MONTH(A57)+1,1)</f>
+        <v>46082</v>
+      </c>
+      <c r="B58" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A58)+IF(MONTH(A58)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C58" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A58,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A58),MONTH(A58)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D58" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A58,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A58),MONTH(A58)+1,1))</f>
+        <v>2048749</v>
+      </c>
+      <c r="F58" s="30">
+        <f>IF(C58="Yes",N(F57)+D58,"")</f>
+        <v>14405730</v>
+      </c>
+      <c r="I58" s="31" t="str">
+        <f>IF(AND(C58="Yes",C59&lt;&gt;"Yes"),B58&amp;" Running Total: "&amp;TEXT(F58,"$0.0,,")&amp;"M (thru "&amp;TEXT(A58,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="28">
+        <f>DATE(YEAR(A58),MONTH(A58)+1,1)</f>
+        <v>46113</v>
+      </c>
+      <c r="B59" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A59)+IF(MONTH(A59)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C59" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A59,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A59),MONTH(A59)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D59" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A59,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A59),MONTH(A59)+1,1))</f>
+        <v>2610208</v>
+      </c>
+      <c r="F59" s="30">
+        <f>IF(C59="Yes",N(F58)+D59,"")</f>
+        <v>17015938</v>
+      </c>
+      <c r="I59" s="31" t="str">
+        <f>IF(AND(C59="Yes",C60&lt;&gt;"Yes"),B59&amp;" Running Total: "&amp;TEXT(F59,"$0.0,,")&amp;"M (thru "&amp;TEXT(A59,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="28">
+        <f>DATE(YEAR(A59),MONTH(A59)+1,1)</f>
+        <v>46143</v>
+      </c>
+      <c r="B60" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A60)+IF(MONTH(A60)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C60" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A60,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A60),MONTH(A60)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D60" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A60,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A60),MONTH(A60)+1,1))</f>
+        <v>2248040</v>
+      </c>
+      <c r="F60" s="30">
+        <f>IF(C60="Yes",N(F59)+D60,"")</f>
+        <v>19263978</v>
+      </c>
+      <c r="I60" s="31" t="str">
+        <f>IF(AND(C60="Yes",C61&lt;&gt;"Yes"),B60&amp;" Running Total: "&amp;TEXT(F60,"$0.0,,")&amp;"M (thru "&amp;TEXT(A60,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="28">
+        <f>DATE(YEAR(A60),MONTH(A60)+1,1)</f>
+        <v>46174</v>
+      </c>
+      <c r="B61" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A61)+IF(MONTH(A61)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C61" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A61,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A61),MONTH(A61)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D61" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A61,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A61),MONTH(A61)+1,1))</f>
+        <v>1772218</v>
+      </c>
+      <c r="F61" s="30">
+        <f>IF(C61="Yes",N(F60)+D61,"")</f>
+        <v>21036196</v>
+      </c>
+      <c r="I61" s="31" t="str">
+        <f>IF(AND(C61="Yes",C62&lt;&gt;"Yes"),B61&amp;" Running Total: "&amp;TEXT(F61,"$0.0,,")&amp;"M (thru "&amp;TEXT(A61,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28">
+        <f>DATE(YEAR(A61),MONTH(A61)+1,1)</f>
+        <v>46204</v>
+      </c>
+      <c r="B62" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A62)+IF(MONTH(A62)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C62" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A62,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A62),MONTH(A62)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D62" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A62,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A62),MONTH(A62)+1,1))</f>
+        <v>2332123</v>
+      </c>
+      <c r="F62" s="30">
+        <f>IF(C62="Yes",N(F61)+D62,"")</f>
+        <v>23368319</v>
+      </c>
+      <c r="I62" s="31" t="str">
+        <f>IF(AND(C62="Yes",C63&lt;&gt;"Yes"),B62&amp;" Running Total: "&amp;TEXT(F62,"$0.0,,")&amp;"M (thru "&amp;TEXT(A62,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="28">
+        <f>DATE(YEAR(A62),MONTH(A62)+1,1)</f>
+        <v>46235</v>
+      </c>
+      <c r="B63" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A63)+IF(MONTH(A63)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C63" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A63,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A63),MONTH(A63)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D63" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A63,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A63),MONTH(A63)+1,1))</f>
+        <v>2450656</v>
+      </c>
+      <c r="F63" s="30">
+        <f>IF(C63="Yes",N(F62)+D63,"")</f>
+        <v>25818975</v>
+      </c>
+      <c r="I63" s="31" t="str">
+        <f>IF(AND(C63="Yes",C64&lt;&gt;"Yes"),B63&amp;" Running Total: "&amp;TEXT(F63,"$0.0,,")&amp;"M (thru "&amp;TEXT(A63,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="28">
+        <f>DATE(YEAR(A63),MONTH(A63)+1,1)</f>
+        <v>46266</v>
+      </c>
+      <c r="B64" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A64)+IF(MONTH(A64)&gt;=10,1,0),2)</f>
+        <v>FY26</v>
+      </c>
+      <c r="C64" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A64,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A64),MONTH(A64)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D64" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A64,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A64),MONTH(A64)+1,1))</f>
+        <v>3524184</v>
+      </c>
+      <c r="F64" s="30">
+        <f>IF(C64="Yes",N(F63)+D64,"")</f>
+        <v>29343159</v>
+      </c>
+      <c r="I64" s="31" t="str">
+        <f>IF(C64="Yes",B64&amp;" Running Total: "&amp;TEXT(F64,"$0.0,,")&amp;"M (thru "&amp;TEXT(A64,"mmm-yy")&amp;")","")</f>
+        <v>FY26 Running Total: $29.3M (thru Sep-26)</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="28">
+        <f>DATE(YEAR(A64),MONTH(A64)+1,1)</f>
+        <v>46296</v>
+      </c>
+      <c r="B65" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A65)+IF(MONTH(A65)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C65" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A65,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A65),MONTH(A65)+1,1))&gt;0,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="D65" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A65,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A65),MONTH(A65)+1,1))</f>
+        <v>2286606</v>
+      </c>
+      <c r="G65" s="30">
+        <f>IF(C65="Yes",D65,"")</f>
+        <v>2286606</v>
+      </c>
+      <c r="J65" s="31" t="str">
+        <f>IF(AND(C65="Yes",C66&lt;&gt;"Yes"),B65&amp;" Running Total: "&amp;TEXT(G65,"$0.0,,")&amp;"M (thru "&amp;TEXT(A65,"mmm-yy")&amp;")","")</f>
+        <v>FY27 Running Total: $2.3M (thru Oct-26)</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="28">
+        <f>DATE(YEAR(A65),MONTH(A65)+1,1)</f>
+        <v>46327</v>
+      </c>
+      <c r="B66" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A66)+IF(MONTH(A66)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C66" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A66,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A66),MONTH(A66)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D66" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A66,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A66),MONTH(A66)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="30" t="str">
+        <f>IF(C66="Yes",N(G65)+D66,"")</f>
+        <v/>
+      </c>
+      <c r="J66" s="31" t="str">
+        <f>IF(AND(C66="Yes",C67&lt;&gt;"Yes"),B66&amp;" Running Total: "&amp;TEXT(G66,"$0.0,,")&amp;"M (thru "&amp;TEXT(A66,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="28">
+        <f>DATE(YEAR(A66),MONTH(A66)+1,1)</f>
+        <v>46357</v>
+      </c>
+      <c r="B67" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A67)+IF(MONTH(A67)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C67" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A67,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A67),MONTH(A67)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D67" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A67,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A67),MONTH(A67)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G67" s="30" t="str">
+        <f>IF(C67="Yes",N(G66)+D67,"")</f>
+        <v/>
+      </c>
+      <c r="J67" s="31" t="str">
+        <f>IF(AND(C67="Yes",C68&lt;&gt;"Yes"),B67&amp;" Running Total: "&amp;TEXT(G67,"$0.0,,")&amp;"M (thru "&amp;TEXT(A67,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="28">
+        <f>DATE(YEAR(A67),MONTH(A67)+1,1)</f>
+        <v>46388</v>
+      </c>
+      <c r="B68" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A68)+IF(MONTH(A68)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C68" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A68,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A68),MONTH(A68)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D68" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A68,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A68),MONTH(A68)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G68" s="30" t="str">
+        <f>IF(C68="Yes",N(G67)+D68,"")</f>
+        <v/>
+      </c>
+      <c r="J68" s="31" t="str">
+        <f>IF(AND(C68="Yes",C69&lt;&gt;"Yes"),B68&amp;" Running Total: "&amp;TEXT(G68,"$0.0,,")&amp;"M (thru "&amp;TEXT(A68,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="28">
+        <f>DATE(YEAR(A68),MONTH(A68)+1,1)</f>
+        <v>46419</v>
+      </c>
+      <c r="B69" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A69)+IF(MONTH(A69)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C69" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A69,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A69),MONTH(A69)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D69" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A69,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A69),MONTH(A69)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G69" s="30" t="str">
+        <f>IF(C69="Yes",N(G68)+D69,"")</f>
+        <v/>
+      </c>
+      <c r="J69" s="31" t="str">
+        <f>IF(AND(C69="Yes",C70&lt;&gt;"Yes"),B69&amp;" Running Total: "&amp;TEXT(G69,"$0.0,,")&amp;"M (thru "&amp;TEXT(A69,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="28">
+        <f>DATE(YEAR(A69),MONTH(A69)+1,1)</f>
+        <v>46447</v>
+      </c>
+      <c r="B70" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A70)+IF(MONTH(A70)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C70" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A70,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A70),MONTH(A70)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D70" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A70,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A70),MONTH(A70)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G70" s="30" t="str">
+        <f>IF(C70="Yes",N(G69)+D70,"")</f>
+        <v/>
+      </c>
+      <c r="J70" s="31" t="str">
+        <f>IF(AND(C70="Yes",C71&lt;&gt;"Yes"),B70&amp;" Running Total: "&amp;TEXT(G70,"$0.0,,")&amp;"M (thru "&amp;TEXT(A70,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="28">
+        <f>DATE(YEAR(A70),MONTH(A70)+1,1)</f>
+        <v>46478</v>
+      </c>
+      <c r="B71" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A71)+IF(MONTH(A71)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C71" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A71,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A71),MONTH(A71)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D71" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A71,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A71),MONTH(A71)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G71" s="30" t="str">
+        <f>IF(C71="Yes",N(G70)+D71,"")</f>
+        <v/>
+      </c>
+      <c r="J71" s="31" t="str">
+        <f>IF(AND(C71="Yes",C72&lt;&gt;"Yes"),B71&amp;" Running Total: "&amp;TEXT(G71,"$0.0,,")&amp;"M (thru "&amp;TEXT(A71,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="28">
+        <f>DATE(YEAR(A71),MONTH(A71)+1,1)</f>
+        <v>46508</v>
+      </c>
+      <c r="B72" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A72)+IF(MONTH(A72)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C72" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A72,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A72),MONTH(A72)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D72" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A72,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A72),MONTH(A72)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G72" s="30" t="str">
+        <f>IF(C72="Yes",N(G71)+D72,"")</f>
+        <v/>
+      </c>
+      <c r="J72" s="31" t="str">
+        <f>IF(AND(C72="Yes",C73&lt;&gt;"Yes"),B72&amp;" Running Total: "&amp;TEXT(G72,"$0.0,,")&amp;"M (thru "&amp;TEXT(A72,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="28">
+        <f>DATE(YEAR(A72),MONTH(A72)+1,1)</f>
+        <v>46539</v>
+      </c>
+      <c r="B73" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A73)+IF(MONTH(A73)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C73" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A73,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A73),MONTH(A73)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D73" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A73,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A73),MONTH(A73)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G73" s="30" t="str">
+        <f>IF(C73="Yes",N(G72)+D73,"")</f>
+        <v/>
+      </c>
+      <c r="J73" s="31" t="str">
+        <f>IF(AND(C73="Yes",C74&lt;&gt;"Yes"),B73&amp;" Running Total: "&amp;TEXT(G73,"$0.0,,")&amp;"M (thru "&amp;TEXT(A73,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="28">
+        <f>DATE(YEAR(A73),MONTH(A73)+1,1)</f>
+        <v>46569</v>
+      </c>
+      <c r="B74" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A74)+IF(MONTH(A74)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C74" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A74,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A74),MONTH(A74)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D74" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A74,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A74),MONTH(A74)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G74" s="30" t="str">
+        <f>IF(C74="Yes",N(G73)+D74,"")</f>
+        <v/>
+      </c>
+      <c r="J74" s="31" t="str">
+        <f>IF(AND(C74="Yes",C75&lt;&gt;"Yes"),B74&amp;" Running Total: "&amp;TEXT(G74,"$0.0,,")&amp;"M (thru "&amp;TEXT(A74,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="28">
+        <f>DATE(YEAR(A74),MONTH(A74)+1,1)</f>
+        <v>46600</v>
+      </c>
+      <c r="B75" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A75)+IF(MONTH(A75)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C75" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A75,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A75),MONTH(A75)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D75" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A75,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A75),MONTH(A75)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G75" s="30" t="str">
+        <f>IF(C75="Yes",N(G74)+D75,"")</f>
+        <v/>
+      </c>
+      <c r="J75" s="31" t="str">
+        <f>IF(AND(C75="Yes",C76&lt;&gt;"Yes"),B75&amp;" Running Total: "&amp;TEXT(G75,"$0.0,,")&amp;"M (thru "&amp;TEXT(A75,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="28">
+        <f>DATE(YEAR(A75),MONTH(A75)+1,1)</f>
+        <v>46631</v>
+      </c>
+      <c r="B76" s="29" t="str">
+        <f>"FY"&amp;RIGHT(YEAR(A76)+IF(MONTH(A76)&gt;=10,1,0),2)</f>
+        <v>FY27</v>
+      </c>
+      <c r="C76" s="29" t="str">
+        <f>IF(COUNTIFS(Metrics!$B$25:$DV$25,"&gt;="&amp;A76,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A76),MONTH(A76)+1,1))&gt;0,"Yes","No")</f>
+        <v>No</v>
+      </c>
+      <c r="D76" s="30">
+        <f>SUMIFS(Metrics!$B$32:$DV$32,Metrics!$B$25:$DV$25,"&gt;="&amp;A76,Metrics!$B$25:$DV$25,"&lt;"&amp;DATE(YEAR(A76),MONTH(A76)+1,1))</f>
+        <v>0</v>
+      </c>
+      <c r="G76" s="30" t="str">
+        <f>IF(C76="Yes",N(G75)+D76,"")</f>
+        <v/>
+      </c>
+      <c r="J76" s="31" t="str">
+        <f>IF(C76="Yes",B76&amp;" Running Total: "&amp;TEXT(G76,"$0.0,,")&amp;"M (thru "&amp;TEXT(A76,"mmm-yy")&amp;")","")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>

</xml_diff>